<commit_message>
Corrige NET do recebimento pela capacidade excedente
</commit_message>
<xml_diff>
--- a/dashboard_local/outputs/01a08633-89b4-7283-8814-f0b65f6970f7/ParametrosOperacionais_Inbound.xlsx
+++ b/dashboard_local/outputs/01a08633-89b4-7283-8814-f0b65f6970f7/ParametrosOperacionais_Inbound.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\performance_geral_cjm\00 - HTML's update\outputs\01a08633-89b4-7283-8814-f0b65f6970f7\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FFC2D04-A627-49B8-8AFA-49F7DDCF8CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3512575-B550-46D8-A87C-45AAFDE1FBA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Orientacoes" sheetId="1" r:id="rId1"/>
@@ -9659,7 +9659,9 @@
       </c>
       <c r="H32" s="76"/>
       <c r="I32" s="82"/>
-      <c r="J32" s="76"/>
+      <c r="J32" s="75">
+        <v>24</v>
+      </c>
       <c r="K32" s="76">
         <v>0</v>
       </c>
@@ -10097,7 +10099,9 @@
       <c r="B17" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C17" s="87"/>
+      <c r="C17" s="87">
+        <v>39</v>
+      </c>
       <c r="D17" s="87">
         <v>257</v>
       </c>
@@ -10106,7 +10110,7 @@
       </c>
       <c r="F17" s="90"/>
       <c r="G17" s="87" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="H17" s="87" t="s">
         <v>282</v>
@@ -10114,7 +10118,7 @@
       <c r="I17" s="87"/>
       <c r="J17" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>NET não calculado</v>
+        <v>NET habilitado</v>
       </c>
       <c r="K17" s="87" t="s">
         <v>256</v>
@@ -14869,14 +14873,14 @@
       <c r="Y30" s="1"/>
       <c r="Z30" s="1"/>
     </row>
-    <row r="31" spans="1:26">
+    <row r="31" spans="1:26" ht="20.25" customHeight="1">
       <c r="A31" s="1" t="s">
         <v>102</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="C31" s="1"/>
+      <c r="C31" s="59"/>
       <c r="D31" s="1">
         <v>40</v>
       </c>
@@ -14915,14 +14919,14 @@
       <c r="Y31" s="1"/>
       <c r="Z31" s="1"/>
     </row>
-    <row r="32" spans="1:26">
+    <row r="32" spans="1:26" ht="34.5" customHeight="1">
       <c r="A32" s="1" t="s">
         <v>106</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C32" s="1"/>
+      <c r="C32" s="59"/>
       <c r="D32" s="1">
         <v>2</v>
       </c>
@@ -14961,14 +14965,14 @@
       <c r="Y32" s="1"/>
       <c r="Z32" s="1"/>
     </row>
-    <row r="33" spans="1:26">
+    <row r="33" spans="1:26" ht="31.5" customHeight="1">
       <c r="A33" s="1" t="s">
         <v>108</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C33" s="1"/>
+      <c r="C33" s="59"/>
       <c r="D33" s="1">
         <v>41</v>
       </c>

</xml_diff>